<commit_message>
Add embed, table-dates blocks, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files: 27
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-naplan.report.xlsx
+++ b/tools/importer/reports/import-naplan.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="88">
   <si>
     <t>_reportFile</t>
   </si>
@@ -52,7 +52,7 @@
     <t>naplan</t>
   </si>
   <si>
-    <t>2026-10-30T04:16:11.050Z</t>
+    <t>2026-10-30T05:37:25.066Z</t>
   </si>
   <si>
     <t>NAP - About</t>
@@ -91,7 +91,7 @@
     <t>nap-sample-assessments</t>
   </si>
   <si>
-    <t>2026-10-30T04:16:18.859Z</t>
+    <t>2026-10-30T05:37:32.176Z</t>
   </si>
   <si>
     <t>NAP sample assessments</t>
@@ -103,7 +103,7 @@
     <t>naplan.report.json</t>
   </si>
   <si>
-    <t>2026-10-30T04:16:25.769Z</t>
+    <t>2026-10-30T05:37:39.813Z</t>
   </si>
   <si>
     <t>NAP - NAPLAN</t>
@@ -121,7 +121,7 @@
     <t>resources</t>
   </si>
   <si>
-    <t>2026-10-30T04:17:18.045Z</t>
+    <t>2026-10-30T05:38:26.772Z</t>
   </si>
   <si>
     <t>Resources</t>
@@ -136,7 +136,7 @@
     <t>results-and-reports</t>
   </si>
   <si>
-    <t>2026-10-30T04:17:25.971Z</t>
+    <t>2026-10-30T05:38:33.047Z</t>
   </si>
   <si>
     <t>Results and reports</t>
@@ -154,7 +154,7 @@
     <t>naplan/faqs</t>
   </si>
   <si>
-    <t>2026-10-30T04:16:30.120Z</t>
+    <t>2026-10-30T05:37:45.679Z</t>
   </si>
   <si>
     <t>NAPLAN - FAQs</t>
@@ -169,7 +169,7 @@
     <t>naplan/for-parents-carers</t>
   </si>
   <si>
-    <t>2026-10-30T04:16:43.686Z</t>
+    <t>2026-10-30T05:37:56.042Z</t>
   </si>
   <si>
     <t>NAP - For parents and carers</t>
@@ -184,7 +184,7 @@
     <t>naplan/for-schools</t>
   </si>
   <si>
-    <t>2026-10-30T04:16:49.747Z</t>
+    <t>2026-10-30T05:38:01.849Z</t>
   </si>
   <si>
     <t>NAP - For schools</t>
@@ -202,7 +202,7 @@
     <t>naplan/key-dates</t>
   </si>
   <si>
-    <t>2026-10-30T04:16:57.901Z</t>
+    <t>2026-10-30T05:38:09.058Z</t>
   </si>
   <si>
     <t>NAP - Key dates</t>
@@ -217,7 +217,7 @@
     <t>naplan/public-demonstration-site</t>
   </si>
   <si>
-    <t>2026-10-30T04:17:04.415Z</t>
+    <t>2026-10-30T05:38:14.984Z</t>
   </si>
   <si>
     <t>NAP - Public demonstration site</t>
@@ -226,13 +226,31 @@
     <t>https://www.nap.edu.au/naplan/public-demonstration-site</t>
   </si>
   <si>
+    <t>naplan/results-and-reports.report.json</t>
+  </si>
+  <si>
+    <t>["cards-side-nav","quote-indented","table-dates","embed"]</t>
+  </si>
+  <si>
+    <t>naplan/results-and-reports</t>
+  </si>
+  <si>
+    <t>2026-10-30T05:38:39.554Z</t>
+  </si>
+  <si>
+    <t>NAPLAN Results and reports</t>
+  </si>
+  <si>
+    <t>https://www.nap.edu.au/naplan/results-and-reports</t>
+  </si>
+  <si>
     <t>naplan/whats-in-the-tests.report.json</t>
   </si>
   <si>
     <t>naplan/whats-in-the-tests</t>
   </si>
   <si>
-    <t>2026-10-30T04:17:10.076Z</t>
+    <t>2026-10-30T05:38:20.379Z</t>
   </si>
   <si>
     <t>NAP - What's in the tests</t>
@@ -250,7 +268,7 @@
     <t>naplan/faqs/naplan-results-reports-performance</t>
   </si>
   <si>
-    <t>2026-10-30T04:16:37.181Z</t>
+    <t>2026-10-30T05:40:43.724Z</t>
   </si>
   <si>
     <t>NAP - NAPLAN - results reports performance</t>
@@ -645,7 +663,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="50" customWidth="1"/>
@@ -973,10 +991,10 @@
         <v>71</v>
       </c>
       <c r="B13" t="s">
-        <v>45</v>
+        <v>72</v>
       </c>
       <c r="C13" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D13" t="s">
         <v>11</v>
@@ -985,21 +1003,21 @@
         <v>12</v>
       </c>
       <c r="F13" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="G13" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="H13" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B14" t="s">
-        <v>77</v>
+        <v>45</v>
       </c>
       <c r="C14" t="s">
         <v>78</v>
@@ -1018,6 +1036,32 @@
       </c>
       <c r="H14" t="s">
         <v>81</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>82</v>
+      </c>
+      <c r="B15" t="s">
+        <v>83</v>
+      </c>
+      <c r="C15" t="s">
+        <v>84</v>
+      </c>
+      <c r="D15" t="s">
+        <v>11</v>
+      </c>
+      <c r="E15" t="s">
+        <v>12</v>
+      </c>
+      <c r="F15" t="s">
+        <v>85</v>
+      </c>
+      <c r="G15" t="s">
+        <v>86</v>
+      </c>
+      <c r="H15" t="s">
+        <v>87</v>
       </c>
     </row>
   </sheetData>

</xml_diff>